<commit_message>
Update scorecards with accurate player and match data
Update scorecards.xlsx to reflect correct scores for Match #52 (Memorial Day) and include player data for Big Foot, CP, Derek Smith, Julian Perico, Kerry Harmon, Nellie, Ty Matlock, and Werner Hugo.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 7fa66303-a6f8-4315-a9eb-c4c029f28cc1
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 278daf8b-8b84-46a9-9d8a-7bdcd90d21fa
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/8e31e601-fae4-4b32-b746-75f14605b3b2/7fa66303-a6f8-4315-a9eb-c4c029f28cc1/G0CzXXd
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/scorecards.xlsx
+++ b/scorecards.xlsx
@@ -1657,7 +1657,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:V17"/>
+  <dimension ref="A1:V26"/>
   <cols>
     <col min="1" max="1" width="20.83203125" customWidth="1"/>
     <col min="2" max="2" width="5.83203125" customWidth="1"/>
@@ -1753,7 +1753,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Chaney</v>
+        <v>Big Foot</v>
       </c>
       <c r="B2">
         <v>4</v>
@@ -1765,84 +1765,84 @@
         <v>5</v>
       </c>
       <c r="E2">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F2">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G2">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H2">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="I2">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J2">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K2">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L2">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M2">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N2">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O2">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="P2">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Q2">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="R2">
         <v>3</v>
       </c>
       <c r="S2">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="T2">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="U2">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="V2">
-        <v>71</v>
+        <v>79</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>Coach</v>
+        <v>CP</v>
       </c>
       <c r="B3">
         <v>5</v>
       </c>
       <c r="C3">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D3">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="E3">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F3">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="G3">
         <v>4</v>
       </c>
       <c r="H3">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="I3">
         <v>4</v>
@@ -1863,16 +1863,16 @@
         <v>4</v>
       </c>
       <c r="O3">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="P3">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Q3">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="R3">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="S3">
         <v>4</v>
@@ -1881,24 +1881,24 @@
         <v>39</v>
       </c>
       <c r="U3">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="V3">
-        <v>73</v>
+        <v>75</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>Cody</v>
+        <v>Chaney</v>
       </c>
       <c r="B4">
         <v>4</v>
       </c>
       <c r="C4">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D4">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E4">
         <v>3</v>
@@ -1913,37 +1913,37 @@
         <v>5</v>
       </c>
       <c r="I4">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J4">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K4">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L4">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="M4">
         <v>4</v>
       </c>
       <c r="N4">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O4">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="P4">
         <v>3</v>
       </c>
       <c r="Q4">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="R4">
         <v>4</v>
       </c>
       <c r="S4">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="T4">
         <v>38</v>
@@ -1957,7 +1957,7 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>DLoe</v>
+        <v>Chip Paris</v>
       </c>
       <c r="B5">
         <v>4</v>
@@ -1969,13 +1969,13 @@
         <v>5</v>
       </c>
       <c r="E5">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F5">
         <v>6</v>
       </c>
       <c r="G5">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H5">
         <v>5</v>
@@ -1984,7 +1984,7 @@
         <v>4</v>
       </c>
       <c r="J5">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K5">
         <v>6</v>
@@ -1993,13 +1993,13 @@
         <v>5</v>
       </c>
       <c r="M5">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N5">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="O5">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="P5">
         <v>3</v>
@@ -2008,101 +2008,101 @@
         <v>5</v>
       </c>
       <c r="R5">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="S5">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="T5">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="U5">
         <v>42</v>
       </c>
       <c r="V5">
-        <v>81</v>
+        <v>84</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>Hot Left Hansson</v>
+        <v>Coach</v>
       </c>
       <c r="B6">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C6">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D6">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E6">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F6">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="G6">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H6">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="I6">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="J6">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="K6">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L6">
         <v>6</v>
       </c>
       <c r="M6">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N6">
         <v>4</v>
       </c>
       <c r="O6">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="P6">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="Q6">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="R6">
         <v>3</v>
       </c>
       <c r="S6">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="T6">
-        <v>34</v>
+        <v>39</v>
       </c>
       <c r="U6">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="V6">
-        <v>72</v>
+        <v>79</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>Hutch</v>
+        <v>Cody</v>
       </c>
       <c r="B7">
         <v>4</v>
       </c>
       <c r="C7">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D7">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="E7">
         <v>3</v>
@@ -2111,10 +2111,10 @@
         <v>4</v>
       </c>
       <c r="G7">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="H7">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="I7">
         <v>4</v>
@@ -2123,93 +2123,93 @@
         <v>5</v>
       </c>
       <c r="K7">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L7">
         <v>5</v>
       </c>
       <c r="M7">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="N7">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="O7">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="P7">
         <v>3</v>
       </c>
       <c r="Q7">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="R7">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="S7">
         <v>4</v>
       </c>
       <c r="T7">
-        <v>42</v>
+        <v>35</v>
       </c>
       <c r="U7">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="V7">
-        <v>82</v>
+        <v>74</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>JP</v>
+        <v>DLoe</v>
       </c>
       <c r="B8">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C8">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D8">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E8">
         <v>3</v>
       </c>
       <c r="F8">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G8">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H8">
         <v>5</v>
       </c>
       <c r="I8">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J8">
         <v>4</v>
       </c>
       <c r="K8">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L8">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M8">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="N8">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O8">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="P8">
         <v>3</v>
       </c>
       <c r="Q8">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="R8">
         <v>3</v>
@@ -2218,10 +2218,10 @@
         <v>4</v>
       </c>
       <c r="T8">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="U8">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="V8">
         <v>76</v>
@@ -2229,16 +2229,16 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>MeerKat</v>
+        <v>Daggs</v>
       </c>
       <c r="B9">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C9">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D9">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E9">
         <v>3</v>
@@ -2247,63 +2247,63 @@
         <v>4</v>
       </c>
       <c r="G9">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H9">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="I9">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J9">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K9">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="L9">
         <v>4</v>
       </c>
       <c r="M9">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N9">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O9">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="P9">
         <v>3</v>
       </c>
       <c r="Q9">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="R9">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="S9">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="T9">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="U9">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="V9">
-        <v>80</v>
+        <v>74</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>Neal</v>
+        <v>Derek Smith</v>
       </c>
       <c r="B10">
         <v>4</v>
       </c>
       <c r="C10">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D10">
         <v>4</v>
@@ -2312,7 +2312,7 @@
         <v>3</v>
       </c>
       <c r="F10">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G10">
         <v>5</v>
@@ -2321,22 +2321,22 @@
         <v>4</v>
       </c>
       <c r="I10">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J10">
         <v>4</v>
       </c>
       <c r="K10">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L10">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M10">
         <v>4</v>
       </c>
       <c r="N10">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O10">
         <v>4</v>
@@ -2348,66 +2348,66 @@
         <v>3</v>
       </c>
       <c r="R10">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="S10">
         <v>4</v>
       </c>
       <c r="T10">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="U10">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="V10">
-        <v>67</v>
+        <v>70</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>Ocker</v>
+        <v>Harrison</v>
       </c>
       <c r="B11">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C11">
         <v>3</v>
       </c>
       <c r="D11">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E11">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="F11">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G11">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H11">
         <v>5</v>
       </c>
       <c r="I11">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="J11">
         <v>5</v>
       </c>
       <c r="K11">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L11">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M11">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="N11">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="O11">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="P11">
         <v>3</v>
@@ -2416,27 +2416,27 @@
         <v>4</v>
       </c>
       <c r="R11">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="S11">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="T11">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="U11">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="V11">
-        <v>74</v>
+        <v>82</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>Sam</v>
+        <v>Hot Left Hansson</v>
       </c>
       <c r="B12">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C12">
         <v>3</v>
@@ -2445,7 +2445,7 @@
         <v>5</v>
       </c>
       <c r="E12">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F12">
         <v>4</v>
@@ -2457,10 +2457,10 @@
         <v>4</v>
       </c>
       <c r="I12">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J12">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K12">
         <v>4</v>
@@ -2469,75 +2469,75 @@
         <v>5</v>
       </c>
       <c r="M12">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N12">
         <v>4</v>
       </c>
       <c r="O12">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="P12">
         <v>3</v>
       </c>
       <c r="Q12">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="R12">
         <v>3</v>
       </c>
       <c r="S12">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="T12">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="U12">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="V12">
-        <v>75</v>
+        <v>70</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>Spikey</v>
+        <v>Hutch</v>
       </c>
       <c r="B13">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C13">
         <v>3</v>
       </c>
       <c r="D13">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E13">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F13">
         <v>5</v>
       </c>
       <c r="G13">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H13">
         <v>4</v>
       </c>
       <c r="I13">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J13">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="K13">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L13">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M13">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="N13">
         <v>4</v>
@@ -2549,95 +2549,95 @@
         <v>3</v>
       </c>
       <c r="Q13">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="R13">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="S13">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="T13">
+        <v>38</v>
+      </c>
+      <c r="U13">
         <v>39</v>
       </c>
-      <c r="U13">
-        <v>36</v>
-      </c>
       <c r="V13">
-        <v>75</v>
+        <v>77</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>Tharnish</v>
+        <v>JP</v>
       </c>
       <c r="B14">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="C14">
         <v>3</v>
       </c>
       <c r="D14">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E14">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F14">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="G14">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H14">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I14">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="J14">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K14">
         <v>5</v>
       </c>
       <c r="L14">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="M14">
         <v>4</v>
       </c>
       <c r="N14">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="O14">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="P14">
         <v>3</v>
       </c>
       <c r="Q14">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="R14">
         <v>4</v>
       </c>
       <c r="S14">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="T14">
-        <v>44</v>
+        <v>37</v>
       </c>
       <c r="U14">
-        <v>44</v>
+        <v>37</v>
       </c>
       <c r="V14">
-        <v>88</v>
+        <v>74</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>Ty Adams</v>
+        <v>Jacob Bartel</v>
       </c>
       <c r="B15">
         <v>4</v>
@@ -2646,66 +2646,66 @@
         <v>3</v>
       </c>
       <c r="D15">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E15">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F15">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G15">
         <v>5</v>
       </c>
       <c r="H15">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="I15">
+        <v>4</v>
+      </c>
+      <c r="J15">
+        <v>3</v>
+      </c>
+      <c r="K15">
+        <v>4</v>
+      </c>
+      <c r="L15">
+        <v>5</v>
+      </c>
+      <c r="M15">
+        <v>4</v>
+      </c>
+      <c r="N15">
+        <v>4</v>
+      </c>
+      <c r="O15">
+        <v>5</v>
+      </c>
+      <c r="P15">
         <v>2</v>
       </c>
-      <c r="J15">
-        <v>4</v>
-      </c>
-      <c r="K15">
-        <v>4</v>
-      </c>
-      <c r="L15">
-        <v>4</v>
-      </c>
-      <c r="M15">
-        <v>5</v>
-      </c>
-      <c r="N15">
-        <v>4</v>
-      </c>
-      <c r="O15">
-        <v>3</v>
-      </c>
-      <c r="P15">
-        <v>3</v>
-      </c>
       <c r="Q15">
         <v>4</v>
       </c>
       <c r="R15">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="S15">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T15">
+        <v>37</v>
+      </c>
+      <c r="U15">
         <v>36</v>
       </c>
-      <c r="U15">
-        <v>33</v>
-      </c>
       <c r="V15">
-        <v>69</v>
+        <v>73</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>Yaffe</v>
+        <v>Julian Perico</v>
       </c>
       <c r="B16">
         <v>4</v>
@@ -2714,99 +2714,99 @@
         <v>3</v>
       </c>
       <c r="D16">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E16">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F16">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G16">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H16">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I16">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J16">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K16">
         <v>5</v>
       </c>
       <c r="L16">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M16">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="N16">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="O16">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="P16">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Q16">
         <v>4</v>
       </c>
       <c r="R16">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="S16">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="T16">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="U16">
-        <v>39</v>
+        <v>32</v>
       </c>
       <c r="V16">
-        <v>74</v>
+        <v>66</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>Zimm</v>
+        <v>Kerry Harmon</v>
       </c>
       <c r="B17">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C17">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D17">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="E17">
         <v>3</v>
       </c>
       <c r="F17">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="G17">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="H17">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="I17">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J17">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="K17">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L17">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M17">
         <v>5</v>
@@ -2815,33 +2815,645 @@
         <v>4</v>
       </c>
       <c r="O17">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="P17">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="Q17">
         <v>4</v>
       </c>
       <c r="R17">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="S17">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="T17">
         <v>39</v>
       </c>
       <c r="U17">
+        <v>41</v>
+      </c>
+      <c r="V17">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>MeerKat</v>
+      </c>
+      <c r="B18">
+        <v>4</v>
+      </c>
+      <c r="C18">
+        <v>3</v>
+      </c>
+      <c r="D18">
+        <v>5</v>
+      </c>
+      <c r="E18">
+        <v>4</v>
+      </c>
+      <c r="F18">
+        <v>4</v>
+      </c>
+      <c r="G18">
+        <v>7</v>
+      </c>
+      <c r="H18">
+        <v>5</v>
+      </c>
+      <c r="I18">
+        <v>4</v>
+      </c>
+      <c r="J18">
+        <v>5</v>
+      </c>
+      <c r="K18">
+        <v>5</v>
+      </c>
+      <c r="L18">
+        <v>5</v>
+      </c>
+      <c r="M18">
+        <v>5</v>
+      </c>
+      <c r="N18">
+        <v>4</v>
+      </c>
+      <c r="O18">
+        <v>4</v>
+      </c>
+      <c r="P18">
+        <v>3</v>
+      </c>
+      <c r="Q18">
+        <v>5</v>
+      </c>
+      <c r="R18">
+        <v>2</v>
+      </c>
+      <c r="S18">
+        <v>6</v>
+      </c>
+      <c r="T18">
+        <v>41</v>
+      </c>
+      <c r="U18">
+        <v>39</v>
+      </c>
+      <c r="V18">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>Neal</v>
+      </c>
+      <c r="B19">
+        <v>4</v>
+      </c>
+      <c r="C19">
+        <v>2</v>
+      </c>
+      <c r="D19">
+        <v>5</v>
+      </c>
+      <c r="E19">
+        <v>3</v>
+      </c>
+      <c r="F19">
+        <v>5</v>
+      </c>
+      <c r="G19">
+        <v>4</v>
+      </c>
+      <c r="H19">
+        <v>4</v>
+      </c>
+      <c r="I19">
+        <v>3</v>
+      </c>
+      <c r="J19">
+        <v>4</v>
+      </c>
+      <c r="K19">
+        <v>5</v>
+      </c>
+      <c r="L19">
+        <v>5</v>
+      </c>
+      <c r="M19">
+        <v>5</v>
+      </c>
+      <c r="N19">
+        <v>4</v>
+      </c>
+      <c r="O19">
+        <v>4</v>
+      </c>
+      <c r="P19">
+        <v>3</v>
+      </c>
+      <c r="Q19">
+        <v>4</v>
+      </c>
+      <c r="R19">
+        <v>3</v>
+      </c>
+      <c r="S19">
+        <v>4</v>
+      </c>
+      <c r="T19">
+        <v>34</v>
+      </c>
+      <c r="U19">
         <v>37</v>
       </c>
-      <c r="V17">
-        <v>76</v>
+      <c r="V19">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>Nellie</v>
+      </c>
+      <c r="B20">
+        <v>4</v>
+      </c>
+      <c r="C20">
+        <v>3</v>
+      </c>
+      <c r="D20">
+        <v>5</v>
+      </c>
+      <c r="E20">
+        <v>4</v>
+      </c>
+      <c r="F20">
+        <v>3</v>
+      </c>
+      <c r="G20">
+        <v>4</v>
+      </c>
+      <c r="H20">
+        <v>4</v>
+      </c>
+      <c r="I20">
+        <v>4</v>
+      </c>
+      <c r="J20">
+        <v>5</v>
+      </c>
+      <c r="K20">
+        <v>6</v>
+      </c>
+      <c r="L20">
+        <v>5</v>
+      </c>
+      <c r="M20">
+        <v>5</v>
+      </c>
+      <c r="N20">
+        <v>4</v>
+      </c>
+      <c r="O20">
+        <v>5</v>
+      </c>
+      <c r="P20">
+        <v>2</v>
+      </c>
+      <c r="Q20">
+        <v>5</v>
+      </c>
+      <c r="R20">
+        <v>5</v>
+      </c>
+      <c r="S20">
+        <v>5</v>
+      </c>
+      <c r="T20">
+        <v>36</v>
+      </c>
+      <c r="U20">
+        <v>42</v>
+      </c>
+      <c r="V20">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>Ocker</v>
+      </c>
+      <c r="B21">
+        <v>4</v>
+      </c>
+      <c r="C21">
+        <v>2</v>
+      </c>
+      <c r="D21">
+        <v>5</v>
+      </c>
+      <c r="E21">
+        <v>3</v>
+      </c>
+      <c r="F21">
+        <v>4</v>
+      </c>
+      <c r="G21">
+        <v>5</v>
+      </c>
+      <c r="H21">
+        <v>4</v>
+      </c>
+      <c r="I21">
+        <v>3</v>
+      </c>
+      <c r="J21">
+        <v>4</v>
+      </c>
+      <c r="K21">
+        <v>5</v>
+      </c>
+      <c r="L21">
+        <v>4</v>
+      </c>
+      <c r="M21">
+        <v>4</v>
+      </c>
+      <c r="N21">
+        <v>5</v>
+      </c>
+      <c r="O21">
+        <v>4</v>
+      </c>
+      <c r="P21">
+        <v>3</v>
+      </c>
+      <c r="Q21">
+        <v>6</v>
+      </c>
+      <c r="R21">
+        <v>3</v>
+      </c>
+      <c r="S21">
+        <v>4</v>
+      </c>
+      <c r="T21">
+        <v>34</v>
+      </c>
+      <c r="U21">
+        <v>38</v>
+      </c>
+      <c r="V21">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>Sam</v>
+      </c>
+      <c r="B22">
+        <v>4</v>
+      </c>
+      <c r="C22">
+        <v>4</v>
+      </c>
+      <c r="D22">
+        <v>4</v>
+      </c>
+      <c r="E22">
+        <v>4</v>
+      </c>
+      <c r="F22">
+        <v>4</v>
+      </c>
+      <c r="G22">
+        <v>5</v>
+      </c>
+      <c r="H22">
+        <v>5</v>
+      </c>
+      <c r="I22">
+        <v>4</v>
+      </c>
+      <c r="J22">
+        <v>5</v>
+      </c>
+      <c r="K22">
+        <v>4</v>
+      </c>
+      <c r="L22">
+        <v>4</v>
+      </c>
+      <c r="M22">
+        <v>4</v>
+      </c>
+      <c r="N22">
+        <v>4</v>
+      </c>
+      <c r="O22">
+        <v>5</v>
+      </c>
+      <c r="P22">
+        <v>3</v>
+      </c>
+      <c r="Q22">
+        <v>4</v>
+      </c>
+      <c r="R22">
+        <v>2</v>
+      </c>
+      <c r="S22">
+        <v>4</v>
+      </c>
+      <c r="T22">
+        <v>39</v>
+      </c>
+      <c r="U22">
+        <v>34</v>
+      </c>
+      <c r="V22">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>Spikey</v>
+      </c>
+      <c r="B23">
+        <v>5</v>
+      </c>
+      <c r="C23">
+        <v>4</v>
+      </c>
+      <c r="D23">
+        <v>6</v>
+      </c>
+      <c r="E23">
+        <v>4</v>
+      </c>
+      <c r="F23">
+        <v>5</v>
+      </c>
+      <c r="G23">
+        <v>4</v>
+      </c>
+      <c r="H23">
+        <v>5</v>
+      </c>
+      <c r="I23">
+        <v>3</v>
+      </c>
+      <c r="J23">
+        <v>4</v>
+      </c>
+      <c r="K23">
+        <v>5</v>
+      </c>
+      <c r="L23">
+        <v>6</v>
+      </c>
+      <c r="M23">
+        <v>4</v>
+      </c>
+      <c r="N23">
+        <v>4</v>
+      </c>
+      <c r="O23">
+        <v>4</v>
+      </c>
+      <c r="P23">
+        <v>4</v>
+      </c>
+      <c r="Q23">
+        <v>4</v>
+      </c>
+      <c r="R23">
+        <v>3</v>
+      </c>
+      <c r="S23">
+        <v>5</v>
+      </c>
+      <c r="T23">
+        <v>40</v>
+      </c>
+      <c r="U23">
+        <v>39</v>
+      </c>
+      <c r="V23">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>Ty Adams</v>
+      </c>
+      <c r="B24">
+        <v>4</v>
+      </c>
+      <c r="C24">
+        <v>3</v>
+      </c>
+      <c r="D24">
+        <v>3</v>
+      </c>
+      <c r="E24">
+        <v>3</v>
+      </c>
+      <c r="F24">
+        <v>6</v>
+      </c>
+      <c r="G24">
+        <v>4</v>
+      </c>
+      <c r="H24">
+        <v>4</v>
+      </c>
+      <c r="I24">
+        <v>3</v>
+      </c>
+      <c r="J24">
+        <v>5</v>
+      </c>
+      <c r="K24">
+        <v>5</v>
+      </c>
+      <c r="L24">
+        <v>4</v>
+      </c>
+      <c r="M24">
+        <v>4</v>
+      </c>
+      <c r="N24">
+        <v>4</v>
+      </c>
+      <c r="O24">
+        <v>5</v>
+      </c>
+      <c r="P24">
+        <v>3</v>
+      </c>
+      <c r="Q24">
+        <v>5</v>
+      </c>
+      <c r="R24">
+        <v>3</v>
+      </c>
+      <c r="S24">
+        <v>4</v>
+      </c>
+      <c r="T24">
+        <v>35</v>
+      </c>
+      <c r="U24">
+        <v>37</v>
+      </c>
+      <c r="V24">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>Ty Matlock</v>
+      </c>
+      <c r="B25">
+        <v>5</v>
+      </c>
+      <c r="C25">
+        <v>2</v>
+      </c>
+      <c r="D25">
+        <v>4</v>
+      </c>
+      <c r="E25">
+        <v>3</v>
+      </c>
+      <c r="F25">
+        <v>6</v>
+      </c>
+      <c r="G25">
+        <v>5</v>
+      </c>
+      <c r="H25">
+        <v>4</v>
+      </c>
+      <c r="I25">
+        <v>4</v>
+      </c>
+      <c r="J25">
+        <v>4</v>
+      </c>
+      <c r="K25">
+        <v>4</v>
+      </c>
+      <c r="L25">
+        <v>3</v>
+      </c>
+      <c r="M25">
+        <v>4</v>
+      </c>
+      <c r="N25">
+        <v>4</v>
+      </c>
+      <c r="O25">
+        <v>6</v>
+      </c>
+      <c r="P25">
+        <v>4</v>
+      </c>
+      <c r="Q25">
+        <v>5</v>
+      </c>
+      <c r="R25">
+        <v>3</v>
+      </c>
+      <c r="S25">
+        <v>4</v>
+      </c>
+      <c r="T25">
+        <v>37</v>
+      </c>
+      <c r="U25">
+        <v>37</v>
+      </c>
+      <c r="V25">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>Werner Hugo</v>
+      </c>
+      <c r="B26">
+        <v>4</v>
+      </c>
+      <c r="C26">
+        <v>3</v>
+      </c>
+      <c r="D26">
+        <v>5</v>
+      </c>
+      <c r="E26">
+        <v>3</v>
+      </c>
+      <c r="F26">
+        <v>5</v>
+      </c>
+      <c r="G26">
+        <v>5</v>
+      </c>
+      <c r="H26">
+        <v>4</v>
+      </c>
+      <c r="I26">
+        <v>4</v>
+      </c>
+      <c r="J26">
+        <v>4</v>
+      </c>
+      <c r="K26">
+        <v>4</v>
+      </c>
+      <c r="L26">
+        <v>4</v>
+      </c>
+      <c r="M26">
+        <v>4</v>
+      </c>
+      <c r="N26">
+        <v>5</v>
+      </c>
+      <c r="O26">
+        <v>4</v>
+      </c>
+      <c r="P26">
+        <v>3</v>
+      </c>
+      <c r="Q26">
+        <v>5</v>
+      </c>
+      <c r="R26">
+        <v>4</v>
+      </c>
+      <c r="S26">
+        <v>4</v>
+      </c>
+      <c r="T26">
+        <v>37</v>
+      </c>
+      <c r="U26">
+        <v>37</v>
+      </c>
+      <c r="V26">
+        <v>74</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:V17"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:V26"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>